<commit_message>
Layout angepast Border auf ein eigene DataTable verschoben
</commit_message>
<xml_diff>
--- a/Werkbank/DataSet/DataTable_Border.xlsx
+++ b/Werkbank/DataSet/DataTable_Border.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\werne\source\repos\KW-Home\CSVtoQR\Werkbank\DataSet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\source\repos\KW-Home\CSVtoQR\Werkbank\DataSet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCCE696E-76C5-4994-B203-CF3D45A5DE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66E5AC7-F94E-47D7-BCAF-712E84FC5C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{EA3B925B-6426-4451-A385-44B0E21C5EF0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA3B925B-6426-4451-A385-44B0E21C5EF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Border" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="7">
-  <si>
-    <t>Stufe</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="10">
   <si>
     <t>Border</t>
   </si>
@@ -57,6 +54,18 @@
   </si>
   <si>
     <t>Top</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>Card</t>
+  </si>
+  <si>
+    <t>Zeile(0)</t>
+  </si>
+  <si>
+    <t>Area</t>
   </si>
 </sst>
 </file>
@@ -166,12 +175,12 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C5A0DDF-543E-4E84-9A4A-A5D1A547EC16}" name="Tabelle8" displayName="Tabelle8" ref="A1:C13" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:C13" xr:uid="{2AD4124C-8309-4C6A-892C-BD298113652A}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B13">
-    <sortCondition ref="A2:A7"/>
-    <sortCondition ref="B2:B7"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C13">
+    <sortCondition ref="A2:A13"/>
+    <sortCondition ref="B2:B13"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{90F62F03-F01E-4C21-B21E-5EBA8D5A97E9}" name="Stufe"/>
+    <tableColumn id="1" xr3:uid="{90F62F03-F01E-4C21-B21E-5EBA8D5A97E9}" name="Area"/>
     <tableColumn id="2" xr3:uid="{B1398070-B2FC-4D45-A220-B5CED81AB8B6}" name="Border"/>
     <tableColumn id="3" xr3:uid="{53CB67DF-F10A-4616-B5EB-AB1E61B5B2AA}" name="Value"/>
   </tableColumns>
@@ -499,8 +508,7 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
@@ -508,142 +516,142 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
       <c r="C5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>0</v>
+      <c r="A6" t="s">
+        <v>7</v>
       </c>
       <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>0</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>0</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>5</v>
       </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>0</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
       <c r="C9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
         <v>3</v>
       </c>
-      <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
         <v>4</v>
       </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
         <v>5</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>6</v>
       </c>
       <c r="C13">
         <v>0</v>

</xml_diff>